<commit_message>
Add quick comment, 20 sample leads, more samples
</commit_message>
<xml_diff>
--- a/sample/more_samples.xlsx
+++ b/sample/more_samples.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leads" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="What each row tests" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -27,17 +28,31 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="005444EC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,15 +60,28 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D5D7E3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -129,6 +157,19 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Leads" displayName="Leads" ref="A1:D21" headerRowCount="1">
+  <autoFilter ref="A1:D21"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Client Name"/>
+    <tableColumn id="2" name="Business Name"/>
+    <tableColumn id="3" name="Post content"/>
+    <tableColumn id="4" name="Email"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -424,12 +465,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="90" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="88" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Client Name</t>
@@ -451,443 +492,716 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Amina Rafiq</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Brew &amp; Bean Cafe</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Opening my cafe next month and need a website with a menu and online reservations. Any recommendations for a good web developer?</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>amina.rafiq@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Hassan Raza</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Raza Auto Parts</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>I want a website for my auto parts shop where customers can browse products. Can anyone recommend a good developer?</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>hassan.raza@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Natalie Brooks</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Brooks Fitness Studio</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Looking for someone to redesign my studio's website. It looks outdated and clients can't book classes online.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>natalie.brooks@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Omar Siddiqui</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Siddiqui Tailors</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Can someone build me a simple website that connects with my Instagram and Facebook pages? Budget is tight.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>omar.siddiqui@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Grace Whitfield</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Whitfield Dental</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Our practice needs a new website with online appointment booking. Who have you used and liked?</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>grace.whitfield@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Daniel Okoye</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Okoye Logistics</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Need a landing page for my new delivery service this week. Fast turnaround please!</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>daniel.okoye@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Sana Tariq</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Sana's Boutique</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Anyone know how to set up an online store for clothes? I'm confused about Shopify vs WordPress.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>sana.tariq@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Marcus Lee</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Lee Plumbing</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Does anyone have a plumber they trust? My sink is leaking again.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>marcus.lee@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Fatima Noor</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Noor Bakes</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Just finished a 3 tier wedding cake order, so proud of the team today!</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>fatima.noor@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Layla Hussain</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Hussain Tutors</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>I want to start online classes. Need a simple website where students can sign up and pay. Suggestions?</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>layla.hussain@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Tom Hardy-Wells</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Wells Landscaping</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>My website got hacked and now shows spam. Need someone who can fix it ASAP.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>tom.wells@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Zainab Ali</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Zainab Henna Art</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Any recommendations for a web designer? I want to show my henna art portfolio online.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>zainab.ali@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Peter Novak</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Novak Photography</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Looking for a web designer who understands photographers. Need a gallery site that loads fast.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>peter.novak@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Rachel Green</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Green Leaf Organics</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Can anyone recommend a good SEO person? My website exists but nobody finds it on Google.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>rachel.green@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Imran Sheikh</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Sheikh Electronics</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>FREE iPhone giveaway!! Click the link and share to win</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>imran.sheikh@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Chloe Bennett</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Bennett Events</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Need a website for my event planning business, nothing fancy, 5 pages max. Budget around $500.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>chloe.bennett@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Ahmed Khan</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Khan Clinic</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Anyone building websites in Karachi? Need one for my clinic.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>ahmed.khan.at.example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Sophie Turner</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Turner Bookkeeping</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Thinking about maybe getting a website someday, not sure yet.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>sophie.turner@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Bilal Hashmi</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Hashmi Catering</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>I need a website with online ordering for my catering business. How long does it usually take?</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>bilal.hashmi@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Ivy Chen</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Ivy's Florals</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Need a florist website with online ordering 🌸 see my page https://facebook.com/ivysflorals</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>ivy.chen@example.com</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="3" t="inlineStr">
+        <is>
+          <t>Business Name</t>
+        </is>
+      </c>
+      <c r="B1" s="3" t="inlineStr">
+        <is>
+          <t>What this row is for</t>
+        </is>
+      </c>
+    </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Amina Rafiq</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Brew &amp; Bean Cafe</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Opening my cafe next month and need a website with a menu and online reservations. Any recommendations for a good web developer?</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>amina.rafiq@example.com</t>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Clear request, strong lead</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Hassan Raza</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Raza Auto Parts</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Mujhe apni shop ki website banwani hai jis mein products ki list ho. Koi achha developer ho to batao.</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>hassan.raza@example.com</t>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Clear request, strong lead</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Natalie Brooks</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Brooks Fitness Studio</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Looking for someone to redesign my studio's website. It looks outdated and clients can't book classes online.</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>natalie.brooks@example.com</t>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Redesign request with a specific problem</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Omar Siddiqui</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>Siddiqui Tailors</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Kya koi mujhe Instagram aur Facebook page ke saath ek simple website bana kar de sakta hai? Budget kam hai.</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>omar.siddiqui@example.com</t>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Budget mention: reply should not invent prices</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Grace Whitfield</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>Whitfield Dental</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Our practice needs a new website with online appointment booking. Who have you used and liked?</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>grace.whitfield@example.com</t>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Asks for recommendations</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Daniel Okoye</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Okoye Logistics</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>Need a landing page for my new delivery service this week. Fast turnaround please!</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>daniel.okoye@example.com</t>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Urgent request</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Sana Tariq</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr">
         <is>
           <t>Sana's Boutique</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Anyone know how to set up an online store for clothes? I'm confused about Shopify vs WordPress.</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>sana.tariq@example.com</t>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Asks a question: a helpful tip fits</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Marcus Lee</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
+      <c r="A9" s="4" t="inlineStr">
         <is>
           <t>Lee Plumbing</t>
         </is>
       </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>Does anyone have a plumber they trust? My sink is leaking again.</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>marcus.lee@example.com</t>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>NOT a lead: should be skipped</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Fatima Noor</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>Noor Bakes</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Just finished a 3 tier wedding cake order, so proud of the team today!</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>fatima.noor@example.com</t>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>NOT a lead: should be skipped</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Layla Hussain</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
+      <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Hussain Tutors</t>
         </is>
       </c>
-      <c r="C11" s="2" t="inlineStr">
-        <is>
-          <t>I want to start online classes. Need a simple website where students can sign up and pay. Suggestions?</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>layla.hussain@example.com</t>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>Clear request with sign-up and payments</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Tom Hardy-Wells</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>Wells Landscaping</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>My website got hacked and now shows spam. Need someone who can fix it ASAP.</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>tom.wells@example.com</t>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>Urgent fix, not a new build</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>Zainab Ali</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
+      <c r="A13" s="4" t="inlineStr">
         <is>
           <t>Zainab Henna Art</t>
         </is>
       </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>Website ke liye koi recommendation? Mujhe apna portfolio online dikhana hai.</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>zainab.ali@example.com</t>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Portfolio site request</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Peter Novak</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
+      <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Novak Photography</t>
         </is>
       </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>Looking for a web designer who understands photographers. Need a gallery site that loads fast.</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>peter.novak@example.com</t>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Specific needs: gallery and speed</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Rachel Green</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>Green Leaf Organics</t>
         </is>
       </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>Can anyone recommend a good SEO person? My website exists but nobody finds it on Google.</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>rachel.green@example.com</t>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Related but not a new build (SEO)</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>Imran Sheikh</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
+      <c r="A16" s="4" t="inlineStr">
         <is>
           <t>Sheikh Electronics</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>FREE iPhone giveaway!! Click the link and share to win</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>imran.sheikh@example.com</t>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>NOT a lead: spam, should be skipped</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Chloe Bennett</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
+      <c r="A17" s="4" t="inlineStr">
         <is>
           <t>Bennett Events</t>
         </is>
       </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>Need a website for my event planning business, nothing fancy, 5 pages max. Budget around $500.</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>chloe.bennett@example.com</t>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>States a budget: reply must not promise a price</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Ahmed Khan</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Khan Clinic</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Anyone building websites in Karachi? Need one for my clinic.</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>ahmed.khan.at.example.com</t>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Invalid email: gets a comment but no email</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Sophie Turner</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
+      <c r="A19" s="4" t="inlineStr">
         <is>
           <t>Turner Bookkeeping</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Thinking about maybe getting a website someday, not sure yet.</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>sophie.turner@example.com</t>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>Low intent: should rank low</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Bilal Hashmi</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
+      <c r="A20" s="4" t="inlineStr">
         <is>
           <t>Hashmi Catering</t>
         </is>
       </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>Catering ke liye online order wali website chahiye. Kitna time lagta hai aam tor par?</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>bilal.hashmi@example.com</t>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>Asks about timing: reply should not promise dates</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>Ivy Chen</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
+      <c r="A21" s="4" t="inlineStr">
         <is>
           <t>Ivy's Florals</t>
         </is>
       </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>Need a florist website with online ordering 🌸 see my page https://facebook.com/ivysflorals</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>ivy.chen@example.com</t>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>Post contains an emoji and a link</t>
         </is>
       </c>
     </row>

</xml_diff>